<commit_message>
Actualización a Versión 1
</commit_message>
<xml_diff>
--- a/datos/ejemplo_ordenes_V1.xlsx
+++ b/datos/ejemplo_ordenes_V1.xlsx
@@ -2,27 +2,30 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
-  <workbookPr/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Katrin\OneDrive\Escritorio\APLICACIONES IA\SCHEDULER\project\datos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/864d67cc60386626/Escritorio/APLICACIONES IA/SCHEDULER/SCHEDULER_V1/datos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A00E52D-41C6-4311-B14E-23B3A56B23B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0B85B02D-F4E3-4DD5-B057-46B738890EF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="15576" windowHeight="9096" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="15576" windowHeight="9096" xr2:uid="{9B58BE8E-27FB-45CC-B436-1D24BD95325D}"/>
   </bookViews>
   <sheets>
-    <sheet name="Ordenes" sheetId="1" r:id="rId1"/>
-    <sheet name="Notas" sheetId="2" r:id="rId2"/>
+    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>id</t>
   </si>
@@ -79,79 +82,13 @@
   </si>
   <si>
     <t>ORD-012</t>
-  </si>
-  <si>
-    <t>Notas sobre el formato de órdenes:</t>
-  </si>
-  <si>
-    <t>COLUMNAS REQUERIDAS:</t>
-  </si>
-  <si>
-    <t>- id: Identificador único de la orden</t>
-  </si>
-  <si>
-    <t>- dim_x: Dimensión X de la pieza en milímetros</t>
-  </si>
-  <si>
-    <t>- dim_y: Dimensión Y de la pieza en milímetros</t>
-  </si>
-  <si>
-    <t>- cantidad: Cantidad a producir</t>
-  </si>
-  <si>
-    <t>- tiempo_unitario: Tiempo de prensado por pieza en horas</t>
-  </si>
-  <si>
-    <t>COLUMNAS OPCIONALES:</t>
-  </si>
-  <si>
-    <t>- presion_psi: Presión de prensado en PSI (para emparejamiento)</t>
-  </si>
-  <si>
-    <t>- prioridad: Nivel de prioridad (1=alta, 5=baja). Default: 3</t>
-  </si>
-  <si>
-    <t>PRENSAS CON PISOS:</t>
-  </si>
-  <si>
-    <t>- P1: 1200x600mm, 50 EUR/h (2 pisos)</t>
-  </si>
-  <si>
-    <t>- P2: 1200x600mm, 50 EUR/h (2 pisos)</t>
-  </si>
-  <si>
-    <t>- P5: 1500x600mm, 60 EUR/h (2 pisos)</t>
-  </si>
-  <si>
-    <t>- P6: 1800x800mm, 75 EUR/h (2 pisos)</t>
-  </si>
-  <si>
-    <t>- P7: 2000x2000mm, 100 EUR/h (2 pisos)</t>
-  </si>
-  <si>
-    <t>RESTRICCIONES DE EMPAREJAMIENTO:</t>
-  </si>
-  <si>
-    <t>- Diferencia máxima de tiempo: 50% del menor tiempo</t>
-  </si>
-  <si>
-    <t>- Diferencia máxima de presión: 20 PSI</t>
-  </si>
-  <si>
-    <t>EJEMPLO DE EMPAREJAMIENTO VÁLIDO:</t>
-  </si>
-  <si>
-    <t>- ORD-001: 1.0 h, 100 PSI con ORD-002: 1.2 h, 110 PSI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  (Diferencia tiempo: 20%, presión: 10 PSI) ✓</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -163,11 +100,6 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -212,7 +144,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -220,13 +152,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -239,7 +170,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -249,44 +180,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F81BD"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="C0504D"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9BBB59"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064A2"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4BACC6"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="F79646"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="800080"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线 Light"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -313,14 +244,32 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -347,6 +296,24 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -358,180 +325,149 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
+                <a:alpha val="63000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+    </a:ext>
+  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B38A57B6-A3E2-4282-90B6-FFA766F87987}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="4" width="10" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="12" customWidth="1"/>
-    <col min="7" max="7" width="10" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -833,129 +769,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:A27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="70" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>40</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>